<commit_message>
Update hazard log Excel (H01 floor transfer, H05 mental health crisis, v0.5 change log) and Evidence base.docx in-place
</commit_message>
<xml_diff>
--- a/docs/clinical-safety/Joint Journey - Hazard Log (DCB0129).xlsx
+++ b/docs/clinical-safety/Joint Journey - Hazard Log (DCB0129).xlsx
@@ -707,7 +707,7 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>"Stop if sharp pain" guidance; "hold onto something sturdy"; "talk to your GP before starting"; gentle/standard/active levelling; warm-up instructions. Pre-exercise safety check collapsible (v0.2). PAR-Q-style safety screening questionnaire during onboarding (v0.4): heart/lung, balance/falls, GP-restricted exercise. Flagged users see persistent caution banner on exercise page.</t>
+          <t>"Stop if sharp pain" guidance; "hold onto something sturdy"; "talk to your GP before starting"; gentle/standard/active levelling; warm-up instructions. Pre-exercise safety check collapsible (v0.2). PAR-Q-style safety screening questionnaire during onboarding (v0.4): heart/lung, balance/falls, GP-restricted exercise. Flagged users see persistent caution banner on exercise page. Floor transfer exercise updated (v0.5, advisory board review Aug 2026): description now advises "try to get up if you feel safe to do so" rather than implying user must always get up. Only attempt if confident; use sturdy chair for support.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>Implemented (v0.4) — screening questionnaire + pre-exercise safety check live.</t>
+          <t>Implemented (v0.5) - screening questionnaire + pre-exercise safety check live; floor transfer wording reviewed by advisory board.</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Evidence-based supportive content. Crisis signposting — persistent "When to seek help" panel surfaces Samaritans 116 123, 111/999, GP routes (v0.2).</t>
+          <t>Evidence-based supportive content. Crisis signposting - persistent "When to seek help" panel surfaces Samaritans 116 123, 111/999, GP routes (v0.2). Explicit mental health crisis entry added (v0.5, advisory board review Aug 2026): call 999 if in immediate danger; call 111 and select mental health option for urgent support. Samaritans entry expanded to include "thoughts of self-harm" and 24/7 availability.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>Implemented (v0.2) — crisis signposting live site-wide.</t>
+          <t>Implemented (v0.5) - crisis signposting live site-wide with explicit mental health crisis routes.</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
@@ -1532,7 +1532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1565,26 +1565,26 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>18/07/2026</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Safety screening questionnaire added to onboarding (PAR-Q-style: heart/lung, balance/falls, exercise restriction). Caution banner on exercise page for flagged users. "Consult your doctor" collapsible added to nutrition page. H01 residual risk reduced to 2×2=4. H04 controls updated, action closed.</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Advisory board review (Aug 2026). H01: Floor transfer exercise wording updated ("try to get up if you feel safe to do so"). H05: Explicit mental health crisis entry added to "When to seek help" panel (999/111 for mental health crises; Samaritans expanded). Content changes: build the bend emphasis, limp timeline (6 months to a year), shower/bath advice, Day 0-1 recovery.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1594,39 +1594,56 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>CSO registered (action closed). Manufacturer updated to Elan Health Ltd (17347255). DPIA cross-reference added to H07 (action closed). H09 and H10 added. Excel hazard log generator created.</t>
+          <t>Safety screening questionnaire added to onboarding (PAR-Q-style: heart/lung, balance/falls, exercise restriction). Caution banner on exercise page for flagged users. "Consult your doctor" collapsible added to nutrition page. H01 residual risk reduced to 2×2=4. H04 controls updated, action closed.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>18/07/2026</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>In-app safety controls implemented: persistent "When to seek help" header control (H02), crisis signposting including Samaritans (H05), pre-exercise safety check (H01).</t>
+          <t>CSO registered (action closed). Manufacturer updated to Elan Health Ltd (17347255). DPIA cross-reference added to H07 (action closed). H09 and H10 added. Excel hazard log generator created.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>In-app safety controls implemented: persistent "When to seek help" header control (H02), crisis signposting including Samaritans (H05), pre-exercise safety check (H01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>29/06/2026</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Initial draft. H01–H08 identified. First-pass risk ratings.</t>
         </is>

</xml_diff>